<commit_message>
BPSpUGBCd, MLfPPR, RPfESCC, STfESCE
</commit_message>
<xml_diff>
--- a/InputData/elec/BPSpUGBCD/BAU Subsidy per Unit Grid Battery Capacity Deployed.xlsx
+++ b/InputData/elec/BPSpUGBCD/BAU Subsidy per Unit Grid Battery Capacity Deployed.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27813"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\elec\BSpUGBCD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ananya.Srinivasan\Documents\EPS\File Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{A50321F0-A6F9-48AB-8C5A-98FD513AF3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C11A953A-C74C-400E-92CD-6962C50867AF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FE9940-7451-4D87-B581-DB68F1A72782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{42D9050D-4015-424A-B242-A22E8EEBF579}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="BPSpUGBCD" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,9 +37,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>BPSpUGBCD BAU Percent Subsidy per Unit Grid Battery Capacity Deployed</t>
+  </si>
+  <si>
+    <t>Dmnl</t>
+  </si>
+  <si>
+    <t>Percent of Capital Cost</t>
   </si>
   <si>
     <t>Source:</t>
@@ -51,42 +57,21 @@
     <t>Notes:</t>
   </si>
   <si>
-    <t xml:space="preserve">In the US version of EPS 4.0, this file assumes developers will opt for the battery ITC, given the </t>
-  </si>
-  <si>
-    <t>incentives in the Inflation Reduction Act. Given the volume of</t>
-  </si>
-  <si>
-    <t>announced battery manufacturing capacity, we assume projects</t>
-  </si>
-  <si>
-    <t>will qualify for the domestic content bonus.</t>
-  </si>
-  <si>
     <t xml:space="preserve">In India, we assume zero subsidies per unit of grid battery capacity although there is an active </t>
   </si>
   <si>
     <t>viability gap fund for battery energy storage. This cannot clearly be expressed as a percentage of subsidy per unit battery capacity</t>
   </si>
-  <si>
-    <t>Dmnl</t>
-  </si>
-  <si>
-    <t>Percent of Capital Cost</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-  </numFmts>
-  <fonts count="6">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -94,32 +79,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -141,13 +101,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -156,13 +111,8 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
-    <cellStyle name="Currency 2" xfId="5" xr:uid="{81BD210F-5FF0-4880-8028-0DC76957F95F}"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 3" xfId="2" xr:uid="{A0D66D47-893E-4339-ABA2-2AA2E8FD27AB}"/>
-    <cellStyle name="Normal 3 2" xfId="3" xr:uid="{6280AA9E-3B50-418D-82DE-98EB684B0878}"/>
-    <cellStyle name="Percent 2" xfId="4" xr:uid="{2FFD538B-3558-46F7-AC70-5718F1F53027}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -178,9 +128,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -188,44 +138,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -253,14 +203,31 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -288,9 +255,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -299,242 +283,214 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
+            <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC948D4D-0473-4A0D-A9E3-0D5B19173DFF}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>3</v>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E25CA65A-E6A8-4244-9C4B-A358863458B6}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AY2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="20.42578125" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:51">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B1">
         <v>2021</v>
@@ -687,9 +643,9 @@
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:51" ht="15.75" customHeight="1">
+    <row r="2" spans="1:51" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -848,17 +804,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A251C7805F896F47A4F48569C73A0799" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="77cd1fc208aa16a525090c2a27f33c66">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f3083de3-5d4e-49f2-a3cd-0aeb079e6739" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d77402130d0e9b5bbfbb66ed18db98d9" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A251C7805F896F47A4F48569C73A0799" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2918bd8377d530163f38b9d795b11f91">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f3083de3-5d4e-49f2-a3cd-0aeb079e6739" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78da601b2f01cef83512fa5499e996db" ns2:_="">
     <xsd:import namespace="f3083de3-5d4e-49f2-a3cd-0aeb079e6739"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -1000,10 +947,29 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1291F06B-7FEA-4994-A08E-346E9CF02F17}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{847B66FF-9742-476E-939C-EE85D107C9F9}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{696F7644-5C3C-4D55-AD09-65FA8A9885EE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFDAB39F-373E-46D2-A502-931EA4CAF472}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A341CAC-1FEE-4EC7-9889-24EF67E2DB07}"/>
 </file>
</xml_diff>